<commit_message>
Graphing in Excel: bar chart example now plots acres; new screenshots; drop stale yield charts
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod_04_bar_chart.xlsx
+++ b/textbook_examples/mod_04_bar_chart.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{FC69407D-4FA9-664C-8568-7461F6F31F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B0D023D-E00D-A842-BA93-37872896762A}"/>
+  <xr:revisionPtr revIDLastSave="260" documentId="8_{FC69407D-4FA9-664C-8568-7461F6F31F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0AAB63E-195F-2C49-8D95-F10F2E9C659D}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="1700" windowWidth="29280" windowHeight="16680" xr2:uid="{1915E7E3-90D0-B946-84B2-001D97E26DFB}"/>
+    <workbookView xWindow="640" yWindow="1700" windowWidth="24780" windowHeight="16680" activeTab="4" xr2:uid="{1915E7E3-90D0-B946-84B2-001D97E26DFB}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="6" r:id="rId1"/>
     <sheet name="Raw data" sheetId="5" r:id="rId2"/>
     <sheet name="All variety bar chart" sheetId="2" r:id="rId3"/>
-    <sheet name="Filtered bar chart" sheetId="4" r:id="rId4"/>
-    <sheet name="Formated bar chart" sheetId="1" r:id="rId5"/>
+    <sheet name="Filtered bar chart" sheetId="8" r:id="rId4"/>
+    <sheet name="Formated bar chart" sheetId="9" r:id="rId5"/>
+    <sheet name="Pie chart" sheetId="7" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All variety bar chart'!$A$1:$C$33</definedName>
@@ -894,11 +895,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'All variety bar chart'!$C$1</c:f>
+              <c:f>'All variety bar chart'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Yield_bu_ac</c:v>
+                  <c:v>Acres</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1019,112 +1020,112 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'All variety bar chart'!$C$2:$C$33</c:f>
+              <c:f>'All variety bar chart'!$B$2:$B$33</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="32"/>
                 <c:pt idx="0">
-                  <c:v>86.6</c:v>
+                  <c:v>392684</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>76.099999999999994</c:v>
+                  <c:v>197626</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>90.1</c:v>
+                  <c:v>143023</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>84.8</c:v>
+                  <c:v>125867</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>88</c:v>
+                  <c:v>74958</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>93.7</c:v>
+                  <c:v>66119</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>48.3</c:v>
+                  <c:v>55767</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>87.4</c:v>
+                  <c:v>38961</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>75.7</c:v>
+                  <c:v>22568</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>77.099999999999994</c:v>
+                  <c:v>21676</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>95.9</c:v>
+                  <c:v>21311</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>96.7</c:v>
+                  <c:v>18710</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>66.900000000000006</c:v>
+                  <c:v>17566</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>40.5</c:v>
+                  <c:v>10249</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>55.9</c:v>
+                  <c:v>8884</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>96</c:v>
+                  <c:v>7282</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>97.1</c:v>
+                  <c:v>6754</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>72.5</c:v>
+                  <c:v>5792</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>102.6</c:v>
+                  <c:v>5636</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>84.1</c:v>
+                  <c:v>5274</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>56.9</c:v>
+                  <c:v>5090</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>73</c:v>
+                  <c:v>4750</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>39.200000000000003</c:v>
+                  <c:v>3015</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>124.7</c:v>
+                  <c:v>2607</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>89.1</c:v>
+                  <c:v>2190</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>97.5</c:v>
+                  <c:v>1998</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>72</c:v>
+                  <c:v>1430</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>56.5</c:v>
+                  <c:v>1287</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>79.2</c:v>
+                  <c:v>901</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>79.2</c:v>
+                  <c:v>825</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>80.099999999999994</c:v>
+                  <c:v>700</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>90.8</c:v>
+                  <c:v>460</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4751-0544-8F59-55FC428F2DE8}"/>
+              <c16:uniqueId val="{00000000-8C01-EF41-BD16-65337E8F1EFB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1138,11 +1139,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="2079362560"/>
-        <c:axId val="2079366592"/>
+        <c:axId val="133457087"/>
+        <c:axId val="133453503"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2079362560"/>
+        <c:axId val="133457087"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1185,7 +1186,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2079366592"/>
+        <c:crossAx val="133453503"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1193,7 +1194,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2079366592"/>
+        <c:axId val="133453503"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1213,7 +1214,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1244,7 +1245,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2079362560"/>
+        <c:crossAx val="133457087"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1348,7 +1349,7 @@
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="col"/>
+        <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
         <c:ser>
@@ -1356,11 +1357,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Filtered bar chart'!$C$1</c:f>
+              <c:f>'Filtered bar chart'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Yield_bu_ac</c:v>
+                  <c:v>Acres</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1381,104 +1382,104 @@
               <c:strCache>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
+                  <c:v>COWBOY CDC</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>RENEGADE CDC</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>ALTORADO</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>LEGACY</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>CLAYMORE</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>ADVANTAGE AB</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>DURANGO CDC</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>MAVERICK CDC</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>CHURCHILL CDC</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>FRASER CDC</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>COPELAND CDC</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>CONNECT AAC</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>AUSTENSON CDC</c:v>
+                </c:pt>
+                <c:pt idx="13">
                   <c:v>SYNERGY AAC</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>AUSTENSON CDC</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>CONNECT AAC</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>COPELAND CDC</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>FRASER CDC</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>CHURCHILL CDC</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>MAVERICK CDC</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>DURANGO CDC</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>ADVANTAGE AB</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>CLAYMORE</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>LEGACY</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>ALTORADO</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>RENEGADE CDC</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>COWBOY CDC</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Filtered bar chart'!$C$2:$C$33</c:f>
+              <c:f>'Filtered bar chart'!$B$2:$B$33</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>86.6</c:v>
+                  <c:v>10249</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>76.099999999999994</c:v>
+                  <c:v>17566</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>90.1</c:v>
+                  <c:v>18710</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>84.8</c:v>
+                  <c:v>21311</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>88</c:v>
+                  <c:v>21676</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>93.7</c:v>
+                  <c:v>22568</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>48.3</c:v>
+                  <c:v>38961</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>87.4</c:v>
+                  <c:v>55767</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>75.7</c:v>
+                  <c:v>66119</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>77.099999999999994</c:v>
+                  <c:v>74958</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>95.9</c:v>
+                  <c:v>125867</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>96.7</c:v>
+                  <c:v>143023</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>66.900000000000006</c:v>
+                  <c:v>197626</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>40.5</c:v>
+                  <c:v>392684</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-951F-BA41-BE1D-09FE9BCAA9F6}"/>
+              <c16:uniqueId val="{00000000-AD85-8545-B9FA-F09A26F95D0F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1491,17 +1492,16 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="2079362560"/>
-        <c:axId val="2079366592"/>
+        <c:axId val="133457087"/>
+        <c:axId val="133453503"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2079362560"/>
+        <c:axId val="133457087"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1539,7 +1539,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2079366592"/>
+        <c:crossAx val="133453503"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1547,12 +1547,12 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2079366592"/>
+        <c:axId val="133453503"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -1567,7 +1567,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1598,7 +1598,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2079362560"/>
+        <c:crossAx val="133457087"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1689,11 +1689,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1600"/>
-              <a:t>Yields</a:t>
+              <a:t>Acres of Barley Varieties</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" sz="1600" baseline="0"/>
-              <a:t> of Barley Varieties in Saskatchewan in 2025</a:t>
+              <a:t> in Saskatchewan in 2025</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="1600"/>
           </a:p>
@@ -1740,19 +1740,19 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Formated bar chart'!$C$1</c:f>
+              <c:f>'Formated bar chart'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Yield_bu_ac</c:v>
+                  <c:v>Acres</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent6">
-                <a:lumMod val="50000"/>
+              <a:schemeClr val="bg2">
+                <a:lumMod val="90000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:ln>
@@ -1761,6 +1761,27 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="10"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-1F38-CC41-BFCE-AA718C693265}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:cat>
             <c:strRef>
               <c:f>'Formated bar chart'!$A$2:$A$33</c:f>
@@ -1770,101 +1791,101 @@
                   <c:v>COWBOY CDC</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>RENEGADE CDC</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>ALTORADO</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>LEGACY</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>CLAYMORE</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>ADVANTAGE AB</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>DURANGO CDC</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>MAVERICK CDC</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>RENEGADE CDC</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>ADVANTAGE AB</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>AUSTENSON CDC</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>CLAYMORE</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>COPELAND CDC</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>SYNERGY AAC</c:v>
-                </c:pt>
                 <c:pt idx="8">
-                  <c:v>DURANGO CDC</c:v>
+                  <c:v>CHURCHILL CDC</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>FRASER CDC</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>COPELAND CDC</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>CONNECT AAC</c:v>
                 </c:pt>
-                <c:pt idx="11">
-                  <c:v>CHURCHILL CDC</c:v>
-                </c:pt>
                 <c:pt idx="12">
-                  <c:v>LEGACY</c:v>
+                  <c:v>AUSTENSON CDC</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>ALTORADO</c:v>
+                  <c:v>SYNERGY AAC</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Formated bar chart'!$C$2:$C$33</c:f>
+              <c:f>'Formated bar chart'!$B$2:$B$33</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>40.5</c:v>
+                  <c:v>10249</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>48.3</c:v>
+                  <c:v>17566</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>66.900000000000006</c:v>
+                  <c:v>18710</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>75.7</c:v>
+                  <c:v>21311</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>76.099999999999994</c:v>
+                  <c:v>21676</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>77.099999999999994</c:v>
+                  <c:v>22568</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>84.8</c:v>
+                  <c:v>38961</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>86.6</c:v>
+                  <c:v>55767</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>87.4</c:v>
+                  <c:v>66119</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>88</c:v>
+                  <c:v>74958</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>90.1</c:v>
+                  <c:v>125867</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>93.7</c:v>
+                  <c:v>143023</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>95.9</c:v>
+                  <c:v>197626</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>96.7</c:v>
+                  <c:v>392684</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3951-D543-AEDC-F71782AB9ADF}"/>
+              <c16:uniqueId val="{00000000-1F38-CC41-BFCE-AA718C693265}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1876,12 +1897,13 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="149"/>
-        <c:axId val="2079362560"/>
-        <c:axId val="2079366592"/>
+        <c:gapWidth val="65"/>
+        <c:overlap val="33"/>
+        <c:axId val="133457087"/>
+        <c:axId val="133453503"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2079362560"/>
+        <c:axId val="133457087"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1924,7 +1946,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2079366592"/>
+        <c:crossAx val="133453503"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1932,11 +1954,10 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2079366592"/>
+        <c:axId val="133453503"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="105"/>
-          <c:min val="0"/>
+          <c:max val="400000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -1961,7 +1982,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -1974,14 +1995,9 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200"/>
-                  <a:t>Average</a:t>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Acres</a:t>
                 </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1200" baseline="0"/>
-                  <a:t> yield (bu/acre)</a:t>
-                </a:r>
-                <a:endParaRPr lang="en-US" sz="1200"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -1998,7 +2014,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -2014,7 +2030,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2045,9 +2061,10 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2079362560"/>
+        <c:crossAx val="133457087"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="100000"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -3734,29 +3751,27 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>266700</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>800100</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9A7895A-D30F-594A-B97E-CA6DEB6AA7C7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D243F905-4048-9FEE-246D-2E222C60FFE1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
+        <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -3777,23 +3792,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>266700</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>660400</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5551A87F-3424-A146-8B13-5E87D6507519}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E6334A2-B7E1-434E-B645-E728718694D8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3820,15 +3835,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>596900</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:colOff>736600</xdr:colOff>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3836,11 +3851,13 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3AB481D-15DA-D361-D375-D1801780DC8E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{145A0403-2AF4-0E47-8988-33D0248C2DA5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -5051,7 +5068,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F60747DF-74A7-C54E-836F-C64742640018}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8B28EB1-3B51-DA44-AA13-C45D848B75C6}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5072,168 +5089,168 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1">
-        <v>392684</v>
+        <v>10249</v>
       </c>
       <c r="C2">
-        <v>86.6</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1">
-        <v>197626</v>
+        <v>17566</v>
       </c>
       <c r="C3">
-        <v>76.099999999999994</v>
+        <v>66.900000000000006</v>
       </c>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1">
-        <v>143023</v>
+        <v>18710</v>
       </c>
       <c r="C4">
-        <v>90.1</v>
+        <v>96.7</v>
       </c>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B5" s="1">
-        <v>125867</v>
+        <v>21311</v>
       </c>
       <c r="C5">
-        <v>84.8</v>
+        <v>95.9</v>
       </c>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1">
-        <v>74958</v>
+        <v>21676</v>
       </c>
       <c r="C6">
-        <v>88</v>
+        <v>77.099999999999994</v>
       </c>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B7" s="1">
-        <v>66119</v>
+        <v>22568</v>
       </c>
       <c r="C7">
-        <v>93.7</v>
+        <v>75.7</v>
       </c>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1">
-        <v>55767</v>
+        <v>38961</v>
       </c>
       <c r="C8">
-        <v>48.3</v>
+        <v>87.4</v>
       </c>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1">
-        <v>38961</v>
+        <v>55767</v>
       </c>
       <c r="C9">
-        <v>87.4</v>
+        <v>48.3</v>
       </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1">
-        <v>22568</v>
+        <v>66119</v>
       </c>
       <c r="C10">
-        <v>75.7</v>
+        <v>93.7</v>
       </c>
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B11" s="1">
-        <v>21676</v>
+        <v>74958</v>
       </c>
       <c r="C11">
-        <v>77.099999999999994</v>
+        <v>88</v>
       </c>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B12" s="1">
-        <v>21311</v>
+        <v>125867</v>
       </c>
       <c r="C12">
-        <v>95.9</v>
+        <v>84.8</v>
       </c>
       <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1">
-        <v>18710</v>
+        <v>143023</v>
       </c>
       <c r="C13">
-        <v>96.7</v>
+        <v>90.1</v>
       </c>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="B14" s="1">
-        <v>17566</v>
+        <v>197626</v>
       </c>
       <c r="C14">
-        <v>66.900000000000006</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1">
-        <v>10249</v>
+        <v>392684</v>
       </c>
       <c r="C15">
-        <v>40.5</v>
+        <v>86.6</v>
       </c>
       <c r="E15" s="1"/>
     </row>
@@ -5460,8 +5477,8 @@
         <customFilter operator="greaterThan" val="10000"/>
       </customFilters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C33">
-      <sortCondition descending="1" ref="B1:B33"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C15">
+      <sortCondition ref="B1:B33"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5470,7 +5487,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45C57125-7BB8-7141-932D-DCCE886206CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{231EA9B6-1BB9-B84A-A87B-2FBFE7F96669}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5502,97 +5519,97 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1">
-        <v>55767</v>
+        <v>17566</v>
       </c>
       <c r="C3">
-        <v>48.3</v>
+        <v>66.900000000000006</v>
       </c>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1">
-        <v>17566</v>
+        <v>18710</v>
       </c>
       <c r="C4">
-        <v>66.900000000000006</v>
+        <v>96.7</v>
       </c>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B5" s="1">
-        <v>22568</v>
+        <v>21311</v>
       </c>
       <c r="C5">
-        <v>75.7</v>
+        <v>95.9</v>
       </c>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1">
-        <v>197626</v>
+        <v>21676</v>
       </c>
       <c r="C6">
-        <v>76.099999999999994</v>
+        <v>77.099999999999994</v>
       </c>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B7" s="1">
-        <v>21676</v>
+        <v>22568</v>
       </c>
       <c r="C7">
-        <v>77.099999999999994</v>
+        <v>75.7</v>
       </c>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1">
-        <v>125867</v>
+        <v>38961</v>
       </c>
       <c r="C8">
-        <v>84.8</v>
+        <v>87.4</v>
       </c>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1">
-        <v>392684</v>
+        <v>55767</v>
       </c>
       <c r="C9">
-        <v>86.6</v>
+        <v>48.3</v>
       </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1">
-        <v>38961</v>
+        <v>66119</v>
       </c>
       <c r="C10">
-        <v>87.4</v>
+        <v>93.7</v>
       </c>
       <c r="E10" s="1"/>
     </row>
@@ -5610,49 +5627,49 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B12" s="1">
-        <v>143023</v>
+        <v>125867</v>
       </c>
       <c r="C12">
-        <v>90.1</v>
+        <v>84.8</v>
       </c>
       <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1">
-        <v>66119</v>
+        <v>143023</v>
       </c>
       <c r="C13">
-        <v>93.7</v>
+        <v>90.1</v>
       </c>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="B14" s="1">
-        <v>21311</v>
+        <v>197626</v>
       </c>
       <c r="C14">
-        <v>95.9</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1">
-        <v>18710</v>
+        <v>392684</v>
       </c>
       <c r="C15">
-        <v>96.7</v>
+        <v>86.6</v>
       </c>
       <c r="E15" s="1"/>
     </row>
@@ -5876,17 +5893,23 @@
   <autoFilter ref="A1:C33" xr:uid="{45C57125-7BB8-7141-932D-DCCE886206CC}">
     <filterColumn colId="1">
       <customFilters>
-        <customFilter operator="greaterThanOrEqual" val="10000"/>
+        <customFilter operator="greaterThan" val="10000"/>
       </customFilters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C15">
-      <sortCondition ref="C1:C33"/>
+      <sortCondition ref="B1:B33"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C33">
-    <sortCondition descending="1" ref="B1:B33"/>
-  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B45BB14C-24F0-3746-9322-48025AF7E09D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Module 4b: shrink chart workbook embeds to two-thirds height; latest workbook saves
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod_04_bar_chart.xlsx
+++ b/textbook_examples/mod_04_bar_chart.xlsx
@@ -8,22 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="8_{FC69407D-4FA9-664C-8568-7461F6F31F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0AAB63E-195F-2C49-8D95-F10F2E9C659D}"/>
+  <xr:revisionPtr revIDLastSave="517" documentId="8_{FC69407D-4FA9-664C-8568-7461F6F31F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E662F1D-82F2-8049-95FF-0AEA9B54F206}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="1700" windowWidth="24780" windowHeight="16680" activeTab="4" xr2:uid="{1915E7E3-90D0-B946-84B2-001D97E26DFB}"/>
+    <workbookView xWindow="640" yWindow="1700" windowWidth="24780" windowHeight="16680" firstSheet="1" activeTab="5" xr2:uid="{1915E7E3-90D0-B946-84B2-001D97E26DFB}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="6" r:id="rId1"/>
     <sheet name="Raw data" sheetId="5" r:id="rId2"/>
-    <sheet name="All variety bar chart" sheetId="2" r:id="rId3"/>
+    <sheet name="Unformated bar chart" sheetId="2" r:id="rId3"/>
     <sheet name="Filtered bar chart" sheetId="8" r:id="rId4"/>
     <sheet name="Formated bar chart" sheetId="9" r:id="rId5"/>
-    <sheet name="Pie chart" sheetId="7" r:id="rId6"/>
+    <sheet name="Unformated pie chart" sheetId="10" r:id="rId6"/>
+    <sheet name="Formated pie chart" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All variety bar chart'!$A$1:$C$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Filtered bar chart'!$A$1:$C$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Formated bar chart'!$A$1:$C$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Unformated bar chart'!$A$1:$C$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Unformated pie chart'!$A$1:$C$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="46">
   <si>
     <t>Variety</t>
   </si>
@@ -178,6 +180,9 @@
   </si>
   <si>
     <t>Formatted horizontal bar chart of yield, sorted low to high, with title "Yields of Barley Varieties in Saskatchewan in 2025"</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -895,7 +900,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'All variety bar chart'!$B$1</c:f>
+              <c:f>'Unformated bar chart'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -916,7 +921,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'All variety bar chart'!$A$2:$A$33</c:f>
+              <c:f>'Unformated bar chart'!$A$2:$A$33</c:f>
               <c:strCache>
                 <c:ptCount val="32"/>
                 <c:pt idx="0">
@@ -1020,7 +1025,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'All variety bar chart'!$B$2:$B$33</c:f>
+              <c:f>'Unformated bar chart'!$B$2:$B$33</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="32"/>
@@ -2118,6 +2123,1374 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Unformated pie chart'!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Acres</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="8"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="9"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="10"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="11"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="12"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="13"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="14"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="15"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="16"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="17"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="18"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="19"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="20"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="21"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="22"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="23"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="24"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="25"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="26"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="27"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="28"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="29"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="30"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="31"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Unformated pie chart'!$A$2:$A$33</c:f>
+              <c:strCache>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>SYNERGY AAC</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>AUSTENSON CDC</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>CONNECT AAC</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>COPELAND CDC</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>FRASER CDC</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>CHURCHILL CDC</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>MAVERICK CDC</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>DURANGO CDC</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>ADVANTAGE AB</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>CLAYMORE</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>LEGACY</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>ALTORADO</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>RENEGADE CDC</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>COWBOY CDC</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>CHAMPION</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>GOLDSTAR CDC</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>ESMA</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>CATTLELAC AB</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>OREANA</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>CONLON</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>METCALFE AC</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>HAGUE AB</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>WRANGLER AB</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>BRAHMA</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>NEWDALE</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>CERVEZA</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>ROSSER AC</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>XENA</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>COPPER CDC</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>MCGWIRE CDC</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>ALBRIGHT AC</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>RATTAN CDC</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Unformated pie chart'!$B$2:$B$33</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>392684</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>197626</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>143023</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>125867</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>74958</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>66119</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>55767</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>38961</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>22568</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>21676</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>21311</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>18710</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>17566</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>10249</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8884</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7282</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>6754</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5792</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5636</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5274</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>5090</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4750</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>3015</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2607</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2190</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1998</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1430</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1287</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>901</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>825</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>460</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3DFC-7447-A983-880E3695BD1D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1800"/>
+              <a:t>Share of Barley Variety Acreage in Saskatchewan 2025</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Formated pie chart'!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Acres</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-D5DB-5A4F-BB1A-79F6AE52FE9F}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-D5DB-5A4F-BB1A-79F6AE52FE9F}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.10648596321393998"/>
+                  <c:y val="9.880239520958084E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="bestFit"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-D5DB-5A4F-BB1A-79F6AE52FE9F}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Formated pie chart'!$A$2:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>SYNERGY AAC</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>AUSTENSON CDC</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>CONNECT AAC</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>COPELAND CDC</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Other</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>FRASER CDC</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>CHURCHILL CDC</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>MAVERICK CDC</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>DURANGO CDC</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>ADVANTAGE AB</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>CLAYMORE</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>LEGACY</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>ALTORADO</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>RENEGADE CDC</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>COWBOY CDC</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>CHAMPION</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>GOLDSTAR CDC</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>ESMA</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>CATTLELAC AB</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>OREANA</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>CONLON</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>METCALFE AC</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>HAGUE AB</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>WRANGLER AB</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>BRAHMA</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>NEWDALE</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>CERVEZA</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>ROSSER AC</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>XENA</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>COPPER CDC</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>MCGWIRE CDC</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>ALBRIGHT AC</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>RATTAN CDC</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Formated pie chart'!$B$2:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>392684</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>197626</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>143023</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>125867</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>412760</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D5DB-5A4F-BB1A-79F6AE52FE9F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="74"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2238,6 +3611,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -3715,6 +5168,1044 @@
             <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -3858,6 +6349,88 @@
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>793750</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>412750</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F925D15-3F93-F4E8-C24D-596C2106C9C3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>184150</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>139700</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E01078F-CA61-F6B9-DCD7-E26DA000491C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -5906,10 +8479,797 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2EE0779-EC26-CD49-AD04-69B0529955D3}">
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="1">
+        <v>392684</v>
+      </c>
+      <c r="C2">
+        <v>86.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1">
+        <v>197626</v>
+      </c>
+      <c r="C3">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1">
+        <v>143023</v>
+      </c>
+      <c r="C4">
+        <v>90.1</v>
+      </c>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1">
+        <v>125867</v>
+      </c>
+      <c r="C5">
+        <v>84.8</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1">
+        <v>74958</v>
+      </c>
+      <c r="C6">
+        <v>88</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1">
+        <v>66119</v>
+      </c>
+      <c r="C7">
+        <v>93.7</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="1">
+        <v>55767</v>
+      </c>
+      <c r="C8">
+        <v>48.3</v>
+      </c>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="1">
+        <v>38961</v>
+      </c>
+      <c r="C9">
+        <v>87.4</v>
+      </c>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1">
+        <v>22568</v>
+      </c>
+      <c r="C10">
+        <v>75.7</v>
+      </c>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="1">
+        <v>21676</v>
+      </c>
+      <c r="C11">
+        <v>77.099999999999994</v>
+      </c>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1">
+        <v>21311</v>
+      </c>
+      <c r="C12">
+        <v>95.9</v>
+      </c>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1">
+        <v>18710</v>
+      </c>
+      <c r="C13">
+        <v>96.7</v>
+      </c>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="1">
+        <v>17566</v>
+      </c>
+      <c r="C14">
+        <v>66.900000000000006</v>
+      </c>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="1">
+        <v>10249</v>
+      </c>
+      <c r="C15">
+        <v>40.5</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="1">
+        <v>8884</v>
+      </c>
+      <c r="C16">
+        <v>55.9</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="1">
+        <v>7282</v>
+      </c>
+      <c r="C17">
+        <v>96</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="1">
+        <v>6754</v>
+      </c>
+      <c r="C18">
+        <v>97.1</v>
+      </c>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="1">
+        <v>5792</v>
+      </c>
+      <c r="C19">
+        <v>72.5</v>
+      </c>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="1">
+        <v>5636</v>
+      </c>
+      <c r="C20">
+        <v>102.6</v>
+      </c>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" s="1">
+        <v>5274</v>
+      </c>
+      <c r="C21">
+        <v>84.1</v>
+      </c>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="1">
+        <v>5090</v>
+      </c>
+      <c r="C22">
+        <v>56.9</v>
+      </c>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>4750</v>
+      </c>
+      <c r="C23">
+        <v>73</v>
+      </c>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="1">
+        <v>3015</v>
+      </c>
+      <c r="C24">
+        <v>39.200000000000003</v>
+      </c>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="1">
+        <v>2607</v>
+      </c>
+      <c r="C25">
+        <v>124.7</v>
+      </c>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="1">
+        <v>2190</v>
+      </c>
+      <c r="C26">
+        <v>89.1</v>
+      </c>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="1">
+        <v>1998</v>
+      </c>
+      <c r="C27">
+        <v>97.5</v>
+      </c>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="1">
+        <v>1430</v>
+      </c>
+      <c r="C28">
+        <v>72</v>
+      </c>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="1">
+        <v>1287</v>
+      </c>
+      <c r="C29">
+        <v>56.5</v>
+      </c>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="1">
+        <v>901</v>
+      </c>
+      <c r="C30">
+        <v>79.2</v>
+      </c>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" s="1">
+        <v>825</v>
+      </c>
+      <c r="C31">
+        <v>79.2</v>
+      </c>
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="1">
+        <v>700</v>
+      </c>
+      <c r="C32">
+        <v>80.099999999999994</v>
+      </c>
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" s="1">
+        <v>460</v>
+      </c>
+      <c r="C33">
+        <v>90.8</v>
+      </c>
+      <c r="E33" s="1"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C33" xr:uid="{45C57125-7BB8-7141-932D-DCCE886206CC}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C33">
+      <sortCondition descending="1" ref="B1:B33"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B45BB14C-24F0-3746-9322-48025AF7E09D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="1">
+        <v>392684</v>
+      </c>
+      <c r="C2">
+        <v>86.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1">
+        <v>197626</v>
+      </c>
+      <c r="C3">
+        <v>76.099999999999994</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1">
+        <v>143023</v>
+      </c>
+      <c r="C4">
+        <v>90.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1">
+        <v>125867</v>
+      </c>
+      <c r="C5">
+        <v>84.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="1">
+        <f>SUM(B8:B35)</f>
+        <v>412760</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="1">
+        <v>74958</v>
+      </c>
+      <c r="C8">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1">
+        <v>66119</v>
+      </c>
+      <c r="C9">
+        <v>93.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="1">
+        <v>55767</v>
+      </c>
+      <c r="C10">
+        <v>48.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1">
+        <v>38961</v>
+      </c>
+      <c r="C11">
+        <v>87.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="1">
+        <v>22568</v>
+      </c>
+      <c r="C12">
+        <v>75.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1">
+        <v>21676</v>
+      </c>
+      <c r="C13">
+        <v>77.099999999999994</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="1">
+        <v>21311</v>
+      </c>
+      <c r="C14">
+        <v>95.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="1">
+        <v>18710</v>
+      </c>
+      <c r="C15">
+        <v>96.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1">
+        <v>17566</v>
+      </c>
+      <c r="C16">
+        <v>66.900000000000006</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1">
+        <v>10249</v>
+      </c>
+      <c r="C17">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="1">
+        <v>8884</v>
+      </c>
+      <c r="C18">
+        <v>55.9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="1">
+        <v>7282</v>
+      </c>
+      <c r="C19">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>6754</v>
+      </c>
+      <c r="C20">
+        <v>97.1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="1">
+        <v>5792</v>
+      </c>
+      <c r="C21">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="1">
+        <v>5636</v>
+      </c>
+      <c r="C22">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="1">
+        <v>5274</v>
+      </c>
+      <c r="C23">
+        <v>84.1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="1">
+        <v>5090</v>
+      </c>
+      <c r="C24">
+        <v>56.9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" s="1">
+        <v>4750</v>
+      </c>
+      <c r="C25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="1">
+        <v>3015</v>
+      </c>
+      <c r="C26">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="1">
+        <v>2607</v>
+      </c>
+      <c r="C27">
+        <v>124.7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>2190</v>
+      </c>
+      <c r="C28">
+        <v>89.1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="1">
+        <v>1998</v>
+      </c>
+      <c r="C29">
+        <v>97.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="1">
+        <v>1430</v>
+      </c>
+      <c r="C30">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="1">
+        <v>1287</v>
+      </c>
+      <c r="C31">
+        <v>56.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="1">
+        <v>901</v>
+      </c>
+      <c r="C32">
+        <v>79.2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="1">
+        <v>825</v>
+      </c>
+      <c r="C33">
+        <v>79.2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" s="1">
+        <v>700</v>
+      </c>
+      <c r="C34">
+        <v>80.099999999999994</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="1">
+        <v>460</v>
+      </c>
+      <c r="C35">
+        <v>90.8</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Two-line chart title: claim only what the chart shows
</commit_message>
<xml_diff>
--- a/textbook_examples/mod_04_bar_chart.xlsx
+++ b/textbook_examples/mod_04_bar_chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="517" documentId="8_{FC69407D-4FA9-664C-8568-7461F6F31F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E662F1D-82F2-8049-95FF-0AEA9B54F206}"/>
+  <xr:revisionPtr revIDLastSave="548" documentId="8_{FC69407D-4FA9-664C-8568-7461F6F31F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BED25B08-06E3-B343-BF71-D8B6D17E50A0}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="1700" windowWidth="24780" windowHeight="16680" firstSheet="1" activeTab="5" xr2:uid="{1915E7E3-90D0-B946-84B2-001D97E26DFB}"/>
+    <workbookView xWindow="640" yWindow="1700" windowWidth="24780" windowHeight="16680" xr2:uid="{1915E7E3-90D0-B946-84B2-001D97E26DFB}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="6" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="50">
   <si>
     <t>Variety</t>
   </si>
@@ -158,38 +158,50 @@
     <t>Raw data</t>
   </si>
   <si>
-    <t>Exploring bar graphs with barley variety data</t>
-  </si>
-  <si>
-    <t>Acres seeded and average yield (bu/ac) for 32 barley varieties, Saskatchewan 2025</t>
-  </si>
-  <si>
-    <t>All variety bar chart</t>
-  </si>
-  <si>
-    <t>Column chart of yield for every variety, unfiltered</t>
-  </si>
-  <si>
     <t>Filtered bar chart</t>
-  </si>
-  <si>
-    <t>Same data with a filter applied so only selected varieties are charted</t>
   </si>
   <si>
     <t>Formated bar chart</t>
   </si>
   <si>
-    <t>Formatted horizontal bar chart of yield, sorted low to high, with title "Yields of Barley Varieties in Saskatchewan in 2025"</t>
+    <t>Other</t>
   </si>
   <si>
-    <t>Other</t>
+    <t>Exploring bar and pie charts with barley variety data</t>
+  </si>
+  <si>
+    <t>Source table: acres seeded and average yield (bu/ac) for 32 barley varieties, Saskatchewan 2025</t>
+  </si>
+  <si>
+    <t>Unformated bar chart</t>
+  </si>
+  <si>
+    <t>Unformated pie chart</t>
+  </si>
+  <si>
+    <t>Formated pie chart</t>
+  </si>
+  <si>
+    <t>Default column chart of acres for all 32 varieties</t>
+  </si>
+  <si>
+    <t>Same chart filtered to the 14 varieties above 10,000 acres</t>
+  </si>
+  <si>
+    <t>The final bar chart</t>
+  </si>
+  <si>
+    <t>Default pie chart of acres for all 32 varieties</t>
+  </si>
+  <si>
+    <t>A formated pie chart</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -342,6 +354,15 @@
     <font>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="14"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -666,32 +687,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -725,6 +720,28 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -773,18 +790,20 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="35" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="12" xfId="42" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="14" xfId="42" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="14" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="12" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -6786,55 +6805,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB00B76-C62D-B340-9872-0E35BDA7B355}">
-  <dimension ref="A3:B10"/>
+  <dimension ref="A3:B12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="73.1640625" customWidth="1"/>
+    <col min="2" max="2" width="92.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="2"/>
+    </row>
+    <row r="6" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="6"/>
+    </row>
+    <row r="7" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="2"/>
-    </row>
-    <row r="6" spans="1:2" ht="19" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="4"/>
-    </row>
-    <row r="7" spans="1:2" ht="19" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="B9" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="19" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="19" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="B10" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B11" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>44</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -6843,9 +6878,11 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A7" location="'Raw data'!A1" tooltip="Go to Raw data" display="Raw data" xr:uid="{1DD753C5-9493-4144-A263-1F462A16B452}"/>
-    <hyperlink ref="A8" location="'All variety bar chart'!A1" tooltip="Go to All variety bar chart" display="All variety bar chart" xr:uid="{6E8969D9-94FD-9F4A-9C0D-10336F23F152}"/>
+    <hyperlink ref="A8" location="'Unformated bar chart'!A1" tooltip="Go to Unformated bar chart" display="Unformated bar chart" xr:uid="{6E8969D9-94FD-9F4A-9C0D-10336F23F152}"/>
     <hyperlink ref="A9" location="'Filtered bar chart'!A1" tooltip="Go to Filtered bar chart" display="Filtered bar chart" xr:uid="{C49EA621-CF9A-C448-B11F-D94EE81038DD}"/>
     <hyperlink ref="A10" location="'Formated bar chart'!A1" tooltip="Go to Formated bar chart" display="Formated bar chart" xr:uid="{F022D751-E233-4E42-99A2-6C2E4A78BA41}"/>
+    <hyperlink ref="A11" location="'Unformated pie chart'!A1" tooltip="Go to Unformated pie chart" display="Unformated pie chart" xr:uid="{95F03E47-25DA-4341-8C00-DE6CB6981711}"/>
+    <hyperlink ref="A12" location="'Formated pie chart'!A1" tooltip="Go to Formated pie chart" display="Formated pie chart" xr:uid="{64FA606B-447E-5B4A-A7D9-BE8843AF10E0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8953,7 +8990,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1">
         <f>SUM(B8:B35)</f>

</xml_diff>